<commit_message>
Add Nigeria/wheat/iron combination with placeholder data (MIC-7549)
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -1404,7 +1404,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="8" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2818,6 +2818,156 @@
         </is>
       </c>
     </row>
+    <row r="29" ht="15" customHeight="1">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Intervention coverage % of fortifiable</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="I29" s="41" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Intervention effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="I30" s="41" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Vehicle fortification in intervention -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>40</v>
+      </c>
+      <c r="J31" s="43" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="4">
     <dataValidation sqref="A1:B1" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1"/>
@@ -2828,7 +2978,7 @@
       <formula1>"Iron,Folate"</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"Bouillon,Salt,Rice"</formula1>
+      <formula1>"Bouillon,Salt,Rice,Wheat"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -2973,7 +3123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M86"/>
+  <dimension ref="A1:M117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="8" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7408,10 +7558,1556 @@
         <v>0.676</v>
       </c>
     </row>
-    <row r="91" ht="15" customHeight="1"/>
-    <row r="92" ht="15" customHeight="1"/>
-    <row r="97" ht="15" customHeight="1"/>
-    <row r="102" ht="15" customHeight="1"/>
+    <row r="87" ht="15" customHeight="1">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Vehicle "fortifiability" (essentially amount industrially produced)</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J87" s="7" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="M87" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="43.5" customHeight="1">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J88" t="n">
+        <v>32.803200000000004</v>
+      </c>
+      <c r="M88" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="43.5" customHeight="1">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J89" t="n">
+        <v>11.491200000000001</v>
+      </c>
+      <c r="M89" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="43.5" customHeight="1">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J90" t="n">
+        <v>23.475200000000001</v>
+      </c>
+      <c r="M90" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="43.5" customHeight="1">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J91" t="n">
+        <v>33.142200000000003</v>
+      </c>
+      <c r="M91" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="43.5" customHeight="1">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J92" t="n">
+        <v>46.652100000000004</v>
+      </c>
+      <c r="M92" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="43.5" customHeight="1">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J93" t="n">
+        <v>53.742000000000004</v>
+      </c>
+      <c r="M93" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="29.25" customHeight="1">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J94" s="21" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="M94" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J95" s="21" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J96" s="21" t="n">
+        <v>0.448</v>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J97" s="21" t="n">
+        <v>0.546</v>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J98" s="21" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J99" s="21" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="29.25" customHeight="1">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J100" t="n">
+        <v>40.074074074074069</v>
+      </c>
+      <c r="M100" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J101" t="n">
+        <v>24.814814814814813</v>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J102" t="n">
+        <v>33.333333333333336</v>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J103" t="n">
+        <v>35.037037037037031</v>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J104" t="n">
+        <v>37.777777777777779</v>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J105" t="n">
+        <v>39.037037037037031</v>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="43.5" customHeight="1">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- amount</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J106" t="n">
+        <v>20.5288</v>
+      </c>
+      <c r="M106" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="43.5" customHeight="1">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- amount</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J107" t="n">
+        <v>19.028000000000002</v>
+      </c>
+      <c r="M107" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="43.5" customHeight="1">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- amount</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J108" t="n">
+        <v>21.976000000000003</v>
+      </c>
+      <c r="M108" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="29.25" customHeight="1">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- amount</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J109" t="n">
+        <v>25.62962962962963</v>
+      </c>
+      <c r="M109" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="29.25" customHeight="1">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- amount</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J110" t="n">
+        <v>23.999999999999996</v>
+      </c>
+      <c r="M110" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="29.25" customHeight="1">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- amount</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J111" t="n">
+        <v>27.333333333333336</v>
+      </c>
+      <c r="M111" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="29.25" customHeight="1">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- any</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J112" s="21" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="M112" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- any</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J113" s="21" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- any</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J114" s="21" t="n">
+        <v>0.448</v>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- any</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J115" s="21" t="n">
+        <v>0.546</v>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- any</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J116" s="21" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- any</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J117" s="21" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="5">
     <dataValidation sqref="A1:B1" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1"/>
@@ -7422,7 +9118,7 @@
       <formula1>"Nigeria,Ethiopia,India"</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"Bouillon,Salt,Rice"</formula1>
+      <formula1>"Bouillon,Salt,Rice,Wheat"</formula1>
     </dataValidation>
     <dataValidation sqref="D1:D1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"All (assumed same),Total,Female,Male"</formula1>
@@ -7939,7 +9635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="8" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9158,11 +10854,161 @@
         </is>
       </c>
     </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- any</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J27" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Baseline effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J28" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="5">
     <dataValidation sqref="A1:B1" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1"/>
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"Bouillon,Salt,Rice"</formula1>
+      <formula1>"Bouillon,Salt,Rice,Wheat"</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Iron,Folate"</formula1>
@@ -11737,7 +13583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="8" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -12011,6 +13857,76 @@
       <c r="I6" s="6" t="inlineStr">
         <is>
           <t>https://www.bmj.com/content/346/bmj.f3443; study of supplementation at higher doses than fortification; selected the effect among trials &lt;66mg/day as all fortification would fall in this range</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="115.5" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Iron fortification/consumption effect on hemoglobin</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Mean difference</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>g/L</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="G7" s="26" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="43.5" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Iron fortification/consumption effect on birthweight</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Mean difference</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>g/(mg/person-day)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct WRA salt SD note; link commits in the test-run log
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ndbs/repos/vivarium_gates_lsff_2026/0100_data_prep/extraction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1576B069-02E3-074B-933C-43694A5BE70D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC47DF2E-8939-6F43-BF05-6887AE0015CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17580" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2176" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2176" uniqueCount="257">
   <si>
     <t>Country</t>
   </si>
@@ -317,9 +317,6 @@
   </si>
   <si>
     <t>Mean per capita salt intake; at 99.3% coverage the among-consumers vs population-mean distinction is immaterial.</t>
-  </si>
-  <si>
-    <t>Assumption: no salt-consumption SD in the GF workbook; CV~0.31 borrowed from the Ethiopia salt extraction (Addis survey SD 2.2 / mean 7.1).</t>
   </si>
   <si>
     <t>GF 'Input data to IHME models' workbook (2026-04-16) (NFCMS 2021), Vehicles - preschool</t>
@@ -1512,28 +1509,28 @@
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>96</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>2</v>
@@ -1579,10 +1576,10 @@
         <v>Complete</v>
       </c>
       <c r="H5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1614,10 +1611,10 @@
         <v>Complete</v>
       </c>
       <c r="H6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1649,10 +1646,10 @@
         <v>Complete</v>
       </c>
       <c r="H7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1684,10 +1681,10 @@
         <v>Complete</v>
       </c>
       <c r="H8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1723,7 +1720,7 @@
         <v>Complete</v>
       </c>
       <c r="I9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1802,62 +1799,62 @@
     </row>
     <row r="3" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" s="44" t="s">
         <v>98</v>
-      </c>
-      <c r="B3" s="44" t="s">
-        <v>99</v>
       </c>
       <c r="C3" s="42"/>
       <c r="D3" s="42"/>
       <c r="E3" s="32" t="s">
+        <v>98</v>
+      </c>
+      <c r="F3" s="32" t="s">
         <v>99</v>
       </c>
-      <c r="F3" s="32" t="s">
-        <v>100</v>
-      </c>
       <c r="G3" s="32" t="s">
+        <v>98</v>
+      </c>
+      <c r="H3" s="32" t="s">
         <v>99</v>
       </c>
-      <c r="H3" s="32" t="s">
-        <v>100</v>
-      </c>
       <c r="I3" s="32" t="s">
+        <v>98</v>
+      </c>
+      <c r="J3" s="33" t="s">
         <v>99</v>
-      </c>
-      <c r="J3" s="33" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="34" t="s">
+        <v>204</v>
+      </c>
+      <c r="B4" s="35" t="s">
         <v>205</v>
       </c>
-      <c r="B4" s="35" t="s">
+      <c r="C4" s="35" t="s">
         <v>206</v>
       </c>
-      <c r="C4" s="35" t="s">
+      <c r="D4" s="36" t="s">
         <v>207</v>
       </c>
-      <c r="D4" s="36" t="s">
+      <c r="E4" s="35" t="s">
         <v>208</v>
       </c>
-      <c r="E4" s="35" t="s">
-        <v>209</v>
-      </c>
       <c r="F4" s="35" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G4" s="35" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H4" s="35" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="I4" s="35" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1871,7 +1868,7 @@
     </row>
     <row r="6" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B6" t="str">
         <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, B$1,  'Scenario Definition Extraction'!$B$2:$B$1000, B$2,  'Scenario Definition Extraction'!$C$2:$C$1000, B$3, 'Scenario Definition Extraction'!$D$2:$D$1000, B$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A6) = 0, "Missing", "Complete")</f>
@@ -1882,7 +1879,7 @@
         <v>Complete</v>
       </c>
       <c r="D6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E6" t="str">
         <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, E$2,  'Scenario Definition Extraction'!$C$2:$C$1000, E$3, 'Scenario Definition Extraction'!$D$2:$D$1000, E$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A6) = 0, "Missing", "Complete")</f>
@@ -1911,7 +1908,7 @@
     </row>
     <row r="7" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B7" t="str">
         <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, B$1,  'Scenario Definition Extraction'!$B$2:$B$1000, B$2,  'Scenario Definition Extraction'!$C$2:$C$1000, B$3, 'Scenario Definition Extraction'!$D$2:$D$1000, B$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A7) = 0, "Missing", "Complete")</f>
@@ -1922,7 +1919,7 @@
         <v>Complete</v>
       </c>
       <c r="D7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E7" t="str">
         <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, E$2,  'Scenario Definition Extraction'!$C$2:$C$1000, E$3, 'Scenario Definition Extraction'!$D$2:$D$1000, E$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A7) = 0, "Missing", "Complete")</f>
@@ -1951,7 +1948,7 @@
     </row>
     <row r="8" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B8" t="str">
         <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, B$1,  'Scenario Definition Extraction'!$B$2:$B$1000, B$2,  'Scenario Definition Extraction'!$C$2:$C$1000, B$3, 'Scenario Definition Extraction'!$D$2:$D$1000, B$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A8) = 0, "Missing", "Complete")</f>
@@ -1962,7 +1959,7 @@
         <v>Complete</v>
       </c>
       <c r="D8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E8" t="str">
         <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, E$2,  'Scenario Definition Extraction'!$C$2:$C$1000, E$3, 'Scenario Definition Extraction'!$D$2:$D$1000, E$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A8) = 0, "Missing", "Complete")</f>
@@ -2031,10 +2028,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -2063,13 +2060,13 @@
         <v>43</v>
       </c>
       <c r="C2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F2" t="s">
         <v>18</v>
@@ -2078,13 +2075,13 @@
         <v>19</v>
       </c>
       <c r="H2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I2" s="37">
         <v>0.71499999999999997</v>
       </c>
       <c r="J2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
@@ -2095,13 +2092,13 @@
         <v>43</v>
       </c>
       <c r="C3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F3" t="s">
         <v>18</v>
@@ -2110,13 +2107,13 @@
         <v>19</v>
       </c>
       <c r="H3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I3" s="37">
         <v>0.71499999999999997</v>
       </c>
       <c r="J3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2127,13 +2124,13 @@
         <v>77</v>
       </c>
       <c r="C4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F4" t="s">
         <v>18</v>
@@ -2142,13 +2139,13 @@
         <v>19</v>
       </c>
       <c r="H4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I4" s="37">
         <v>0.95</v>
       </c>
       <c r="J4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
@@ -2159,13 +2156,13 @@
         <v>77</v>
       </c>
       <c r="C5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F5" t="s">
         <v>18</v>
@@ -2174,13 +2171,13 @@
         <v>19</v>
       </c>
       <c r="H5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I5" s="37">
         <v>0.95</v>
       </c>
       <c r="J5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
@@ -2191,13 +2188,13 @@
         <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F6" t="s">
         <v>18</v>
@@ -2206,13 +2203,13 @@
         <v>19</v>
       </c>
       <c r="H6" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="I6" s="37">
         <v>0.95</v>
       </c>
       <c r="J6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
@@ -2223,13 +2220,13 @@
         <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F7" t="s">
         <v>18</v>
@@ -2238,13 +2235,13 @@
         <v>19</v>
       </c>
       <c r="H7" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="I7" s="37">
         <v>0.95</v>
       </c>
       <c r="J7" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
@@ -2255,13 +2252,13 @@
         <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F8" t="s">
         <v>18</v>
@@ -2270,13 +2267,13 @@
         <v>19</v>
       </c>
       <c r="H8" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="I8" s="37">
         <v>0.95</v>
       </c>
       <c r="J8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
@@ -2287,13 +2284,13 @@
         <v>77</v>
       </c>
       <c r="C9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E9" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F9" t="s">
         <v>18</v>
@@ -2302,13 +2299,13 @@
         <v>19</v>
       </c>
       <c r="H9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I9" s="37">
         <v>0.92</v>
       </c>
       <c r="J9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
@@ -2319,13 +2316,13 @@
         <v>77</v>
       </c>
       <c r="C10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D10" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E10" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F10" t="s">
         <v>18</v>
@@ -2334,13 +2331,13 @@
         <v>19</v>
       </c>
       <c r="H10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I10" s="37">
         <v>0.92</v>
       </c>
       <c r="J10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
@@ -2351,13 +2348,13 @@
         <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D11" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F11" t="s">
         <v>18</v>
@@ -2366,13 +2363,13 @@
         <v>19</v>
       </c>
       <c r="H11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I11" s="37">
         <v>0.71499999999999997</v>
       </c>
       <c r="J11" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
@@ -2383,13 +2380,13 @@
         <v>43</v>
       </c>
       <c r="C12" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D12" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E12" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F12" t="s">
         <v>18</v>
@@ -2398,13 +2395,13 @@
         <v>19</v>
       </c>
       <c r="H12" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I12" s="37">
         <v>0.71499999999999997</v>
       </c>
       <c r="J12" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2415,13 +2412,13 @@
         <v>77</v>
       </c>
       <c r="C13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D13" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E13" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F13" t="s">
         <v>18</v>
@@ -2430,13 +2427,13 @@
         <v>19</v>
       </c>
       <c r="H13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I13" s="37">
         <v>0.95</v>
       </c>
       <c r="J13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
@@ -2447,13 +2444,13 @@
         <v>77</v>
       </c>
       <c r="C14" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D14" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E14" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F14" t="s">
         <v>18</v>
@@ -2462,13 +2459,13 @@
         <v>19</v>
       </c>
       <c r="H14" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I14" s="37">
         <v>0.95</v>
       </c>
       <c r="J14" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
@@ -2479,13 +2476,13 @@
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D15" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E15" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F15" t="s">
         <v>18</v>
@@ -2494,13 +2491,13 @@
         <v>19</v>
       </c>
       <c r="H15" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="I15" s="37">
         <v>0.95</v>
       </c>
       <c r="J15" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
@@ -2511,13 +2508,13 @@
         <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D16" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E16" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F16" t="s">
         <v>18</v>
@@ -2526,13 +2523,13 @@
         <v>19</v>
       </c>
       <c r="H16" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="I16" s="37">
         <v>0.95</v>
       </c>
       <c r="J16" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
@@ -2543,13 +2540,13 @@
         <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D17" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E17" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>
@@ -2558,13 +2555,13 @@
         <v>19</v>
       </c>
       <c r="H17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="I17" s="37">
         <v>0.95</v>
       </c>
       <c r="J17" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2575,13 +2572,13 @@
         <v>77</v>
       </c>
       <c r="C18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D18" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E18" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F18" t="s">
         <v>18</v>
@@ -2590,13 +2587,13 @@
         <v>19</v>
       </c>
       <c r="H18" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I18" s="37">
         <v>0.92</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2607,13 +2604,13 @@
         <v>77</v>
       </c>
       <c r="C19" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D19" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E19" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F19" t="s">
         <v>18</v>
@@ -2622,13 +2619,13 @@
         <v>19</v>
       </c>
       <c r="H19" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I19" s="37">
         <v>0.92</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -2639,28 +2636,28 @@
         <v>43</v>
       </c>
       <c r="C20" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D20" t="s">
+        <v>208</v>
+      </c>
+      <c r="E20" t="s">
         <v>209</v>
       </c>
-      <c r="E20" t="s">
-        <v>210</v>
-      </c>
       <c r="F20" t="s">
+        <v>106</v>
+      </c>
+      <c r="G20" t="s">
         <v>107</v>
       </c>
-      <c r="G20" t="s">
-        <v>108</v>
-      </c>
       <c r="H20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="I20">
         <v>1320</v>
       </c>
       <c r="J20" s="38" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -2671,28 +2668,28 @@
         <v>43</v>
       </c>
       <c r="C21" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D21" t="s">
+        <v>208</v>
+      </c>
+      <c r="E21" t="s">
         <v>209</v>
       </c>
-      <c r="E21" t="s">
-        <v>210</v>
-      </c>
       <c r="F21" t="s">
+        <v>106</v>
+      </c>
+      <c r="G21" t="s">
         <v>107</v>
       </c>
-      <c r="G21" t="s">
-        <v>108</v>
-      </c>
       <c r="H21" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="I21">
         <v>24</v>
       </c>
       <c r="J21" s="38" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
@@ -2703,28 +2700,28 @@
         <v>77</v>
       </c>
       <c r="C22" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D22" t="s">
+        <v>208</v>
+      </c>
+      <c r="E22" t="s">
         <v>209</v>
       </c>
-      <c r="E22" t="s">
-        <v>210</v>
-      </c>
       <c r="F22" t="s">
+        <v>106</v>
+      </c>
+      <c r="G22" t="s">
         <v>107</v>
       </c>
-      <c r="G22" t="s">
-        <v>108</v>
-      </c>
       <c r="H22" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="I22">
         <v>40</v>
       </c>
       <c r="J22" s="39" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
@@ -2735,28 +2732,28 @@
         <v>77</v>
       </c>
       <c r="C23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D23" t="s">
+        <v>208</v>
+      </c>
+      <c r="E23" t="s">
         <v>209</v>
       </c>
-      <c r="E23" t="s">
-        <v>210</v>
-      </c>
       <c r="F23" t="s">
+        <v>106</v>
+      </c>
+      <c r="G23" t="s">
         <v>107</v>
       </c>
-      <c r="G23" t="s">
-        <v>108</v>
-      </c>
       <c r="H23" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="I23">
         <v>1.69</v>
       </c>
       <c r="J23" s="39" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
@@ -2767,28 +2764,28 @@
         <v>14</v>
       </c>
       <c r="C24" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D24" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E24" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F24" t="s">
+        <v>106</v>
+      </c>
+      <c r="G24" t="s">
         <v>107</v>
       </c>
-      <c r="G24" t="s">
-        <v>108</v>
-      </c>
       <c r="H24" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="I24">
         <v>14.08450704225352</v>
       </c>
       <c r="J24" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2799,28 +2796,28 @@
         <v>14</v>
       </c>
       <c r="C25" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D25" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E25" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F25" t="s">
+        <v>106</v>
+      </c>
+      <c r="G25" t="s">
         <v>107</v>
       </c>
-      <c r="G25" t="s">
-        <v>108</v>
-      </c>
       <c r="H25" s="40" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="I25">
         <v>56.338028169014088</v>
       </c>
       <c r="J25" s="40" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
@@ -2831,28 +2828,28 @@
         <v>14</v>
       </c>
       <c r="C26" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D26" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E26" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F26" t="s">
+        <v>106</v>
+      </c>
+      <c r="G26" t="s">
         <v>107</v>
       </c>
-      <c r="G26" t="s">
-        <v>108</v>
-      </c>
       <c r="H26" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I26">
         <v>45</v>
       </c>
       <c r="J26" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
@@ -2863,28 +2860,28 @@
         <v>77</v>
       </c>
       <c r="C27" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D27" t="s">
+        <v>208</v>
+      </c>
+      <c r="E27" t="s">
         <v>209</v>
       </c>
-      <c r="E27" t="s">
-        <v>210</v>
-      </c>
       <c r="F27" t="s">
+        <v>106</v>
+      </c>
+      <c r="G27" t="s">
         <v>107</v>
       </c>
-      <c r="G27" t="s">
-        <v>108</v>
-      </c>
       <c r="H27" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="I27">
         <v>42.5</v>
       </c>
       <c r="J27" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
@@ -2895,28 +2892,28 @@
         <v>77</v>
       </c>
       <c r="C28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D28" t="s">
+        <v>208</v>
+      </c>
+      <c r="E28" t="s">
         <v>209</v>
       </c>
-      <c r="E28" t="s">
-        <v>210</v>
-      </c>
       <c r="F28" t="s">
+        <v>106</v>
+      </c>
+      <c r="G28" t="s">
         <v>107</v>
       </c>
-      <c r="G28" t="s">
-        <v>108</v>
-      </c>
       <c r="H28" s="39" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="I28">
         <v>1.3</v>
       </c>
       <c r="J28" s="39" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
@@ -2927,13 +2924,13 @@
         <v>14</v>
       </c>
       <c r="C29" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D29" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E29" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F29" t="s">
         <v>18</v>
@@ -2942,13 +2939,13 @@
         <v>19</v>
       </c>
       <c r="H29" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="I29">
         <v>0.95</v>
       </c>
       <c r="J29" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
@@ -2959,13 +2956,13 @@
         <v>14</v>
       </c>
       <c r="C30" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D30" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E30" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F30" t="s">
         <v>18</v>
@@ -2974,13 +2971,13 @@
         <v>19</v>
       </c>
       <c r="H30" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="I30">
         <v>0.95</v>
       </c>
       <c r="J30" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
@@ -2991,28 +2988,28 @@
         <v>14</v>
       </c>
       <c r="C31" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D31" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E31" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F31" t="s">
+        <v>106</v>
+      </c>
+      <c r="G31" t="s">
         <v>107</v>
       </c>
-      <c r="G31" t="s">
-        <v>108</v>
-      </c>
       <c r="H31" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I31">
         <v>25.641025641025639</v>
       </c>
       <c r="J31" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
@@ -3023,13 +3020,13 @@
         <v>14</v>
       </c>
       <c r="C32" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D32" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E32" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F32" t="s">
         <v>18</v>
@@ -3038,13 +3035,13 @@
         <v>19</v>
       </c>
       <c r="H32" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="I32">
         <v>0.95</v>
       </c>
       <c r="J32" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
@@ -3055,13 +3052,13 @@
         <v>14</v>
       </c>
       <c r="C33" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D33" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E33" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F33" t="s">
         <v>18</v>
@@ -3070,13 +3067,13 @@
         <v>19</v>
       </c>
       <c r="H33" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="I33">
         <v>0.95</v>
       </c>
       <c r="J33" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
@@ -3087,28 +3084,28 @@
         <v>14</v>
       </c>
       <c r="C34" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D34" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E34" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F34" t="s">
+        <v>106</v>
+      </c>
+      <c r="G34" t="s">
         <v>107</v>
       </c>
-      <c r="G34" t="s">
-        <v>108</v>
-      </c>
       <c r="H34" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I34">
         <v>102.5641025641026</v>
       </c>
       <c r="J34" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -3296,22 +3293,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>244</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>245</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -3319,13 +3316,13 @@
         <v>44</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>46</v>
       </c>
       <c r="D2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E2">
         <v>2021</v>
@@ -3333,30 +3330,30 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>248</v>
+      </c>
+      <c r="B3" t="s">
         <v>249</v>
-      </c>
-      <c r="B3" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>250</v>
+      </c>
+      <c r="B4" t="s">
         <v>251</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" t="s">
         <v>253</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" s="16" t="s">
         <v>254</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="F4" t="s">
         <v>255</v>
-      </c>
-      <c r="F4" t="s">
-        <v>256</v>
       </c>
     </row>
   </sheetData>
@@ -6710,7 +6707,7 @@
         <v>1.21</v>
       </c>
       <c r="M99" t="s">
-        <v>91</v>
+        <v>256</v>
       </c>
     </row>
     <row r="100" spans="1:13" x14ac:dyDescent="0.2">
@@ -6884,7 +6881,7 @@
         <v>2021</v>
       </c>
       <c r="I105" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J105">
         <v>0.99</v>
@@ -6916,7 +6913,7 @@
         <v>2021</v>
       </c>
       <c r="I106" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J106">
         <v>2.6</v>
@@ -6948,7 +6945,7 @@
         <v>2021</v>
       </c>
       <c r="I107" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J107">
         <v>2.5</v>
@@ -6980,7 +6977,7 @@
         <v>2021</v>
       </c>
       <c r="I108" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J108">
         <v>2.7</v>
@@ -7015,7 +7012,7 @@
         <v>0.81</v>
       </c>
       <c r="M109" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="110" spans="1:13" x14ac:dyDescent="0.2">
@@ -7044,13 +7041,13 @@
         <v>2026</v>
       </c>
       <c r="I110" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J110">
         <v>0.95</v>
       </c>
       <c r="M110" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="111" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -8699,89 +8696,89 @@
     </row>
     <row r="3" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" s="41" t="s">
         <v>98</v>
-      </c>
-      <c r="B3" s="41" t="s">
-        <v>99</v>
       </c>
       <c r="C3" s="42"/>
       <c r="D3" s="41" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E3" s="42"/>
       <c r="F3" s="41" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G3" s="42"/>
       <c r="H3" s="41" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I3" s="42"/>
       <c r="J3" s="41" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K3" s="42"/>
       <c r="L3" s="41" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M3" s="42"/>
       <c r="N3" s="41" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="O3" s="42"/>
       <c r="P3" s="41" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q3" s="42"/>
     </row>
     <row r="4" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>96</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="O4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="Q4" s="1" t="s">
         <v>2</v>
@@ -8800,25 +8797,25 @@
     </row>
     <row r="6" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B6" t="s">
         <v>101</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D6" t="s">
         <v>102</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
         <v>102</v>
       </c>
-      <c r="D6" t="s">
-        <v>103</v>
-      </c>
-      <c r="E6" t="s">
-        <v>103</v>
-      </c>
       <c r="F6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H6" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$944, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$944, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$944, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$944, "Total",  'Country-Vehicle-Fort Extraction'!$E$2:$E$944, $A6, 'Country-Vehicle-Fort Extraction'!$J$2:$J$944, "&lt;&gt;") = 0, "Missing", "Complete")</f>
@@ -8829,51 +8826,51 @@
         <v>Complete</v>
       </c>
       <c r="J6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="K6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="O6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="Q6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" t="s">
+        <v>101</v>
+      </c>
+      <c r="D7" t="s">
         <v>102</v>
       </c>
-      <c r="C7" t="s">
+      <c r="E7" t="s">
         <v>102</v>
       </c>
-      <c r="D7" t="s">
-        <v>103</v>
-      </c>
-      <c r="E7" t="s">
-        <v>103</v>
-      </c>
       <c r="F7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H7" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$944, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$944, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$944, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$944, "Total",  'Country-Vehicle-Fort Extraction'!$E$2:$E$944, $A7, 'Country-Vehicle-Fort Extraction'!$J$2:$J$944, "&lt;&gt;") = 0, "Missing", "Complete")</f>
@@ -8884,53 +8881,53 @@
         <v>Missing</v>
       </c>
       <c r="J7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="K7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N7" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$944, N$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$944, N$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$944, N$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$944, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$944, $A7, 'Country-Vehicle-Fort Extraction'!$J$2:$J$944, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="O7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="P7" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$944, N$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$944, N$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$944, P$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$944, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$944, $A7, 'Country-Vehicle-Fort Extraction'!$J$2:$J$944, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="Q7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B8" t="s">
+        <v>101</v>
+      </c>
+      <c r="C8" t="s">
+        <v>101</v>
+      </c>
+      <c r="D8" t="s">
         <v>102</v>
       </c>
-      <c r="C8" t="s">
+      <c r="E8" t="s">
         <v>102</v>
       </c>
-      <c r="D8" t="s">
-        <v>103</v>
-      </c>
-      <c r="E8" t="s">
-        <v>103</v>
-      </c>
       <c r="F8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H8" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$944, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$944, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$944, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$944, "Total",  'Country-Vehicle-Fort Extraction'!$E$2:$E$944, $A8, 'Country-Vehicle-Fort Extraction'!$J$2:$J$944, "&lt;&gt;") = 0, "Missing", "Complete")</f>
@@ -8941,30 +8938,30 @@
         <v>Missing</v>
       </c>
       <c r="J8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="K8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N8" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$944, N$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$944, N$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$944, N$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$944, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$944, $A8, 'Country-Vehicle-Fort Extraction'!$J$2:$J$944, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="O8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="P8" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$944, N$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$944, N$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$944, P$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$944, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$944, $A8, 'Country-Vehicle-Fort Extraction'!$J$2:$J$944, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="Q8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -9021,7 +9018,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -9059,13 +9056,13 @@
         <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D2" t="s">
         <v>15</v>
       </c>
       <c r="E2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F2" t="s">
         <v>18</v>
@@ -9088,19 +9085,19 @@
         <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D3" t="s">
         <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G3" s="8" t="s">
         <v>107</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>108</v>
       </c>
       <c r="I3" t="s">
         <v>40</v>
@@ -9117,13 +9114,13 @@
         <v>77</v>
       </c>
       <c r="C4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D4" t="s">
         <v>15</v>
       </c>
       <c r="E4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F4" t="s">
         <v>18</v>
@@ -9138,7 +9135,7 @@
         <v>0</v>
       </c>
       <c r="L4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -9149,19 +9146,19 @@
         <v>77</v>
       </c>
       <c r="C5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D5" t="s">
         <v>15</v>
       </c>
       <c r="E5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F5" t="s">
+        <v>106</v>
+      </c>
+      <c r="G5" s="8" t="s">
         <v>107</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>108</v>
       </c>
       <c r="I5" t="s">
         <v>40</v>
@@ -9170,7 +9167,7 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -9181,13 +9178,13 @@
         <v>77</v>
       </c>
       <c r="C6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D6" t="s">
         <v>15</v>
       </c>
       <c r="E6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F6" t="s">
         <v>18</v>
@@ -9202,7 +9199,7 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -9213,19 +9210,19 @@
         <v>77</v>
       </c>
       <c r="C7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D7" t="s">
         <v>15</v>
       </c>
       <c r="E7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F7" t="s">
+        <v>106</v>
+      </c>
+      <c r="G7" s="8" t="s">
         <v>107</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>108</v>
       </c>
       <c r="I7" t="s">
         <v>40</v>
@@ -9234,7 +9231,7 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
@@ -9245,13 +9242,13 @@
         <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D8" t="s">
         <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F8" t="s">
         <v>18</v>
@@ -9266,7 +9263,7 @@
         <v>0.61875637104994896</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
@@ -9277,13 +9274,13 @@
         <v>43</v>
       </c>
       <c r="C9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D9" t="s">
         <v>27</v>
       </c>
       <c r="E9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F9" t="s">
         <v>18</v>
@@ -9307,13 +9304,13 @@
         <v>43</v>
       </c>
       <c r="C10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D10" t="s">
         <v>28</v>
       </c>
       <c r="E10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F10" t="s">
         <v>18</v>
@@ -9337,13 +9334,13 @@
         <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D11" t="s">
         <v>29</v>
       </c>
       <c r="E11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F11" t="s">
         <v>18</v>
@@ -9367,13 +9364,13 @@
         <v>43</v>
       </c>
       <c r="C12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D12" t="s">
         <v>30</v>
       </c>
       <c r="E12" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F12" t="s">
         <v>18</v>
@@ -9397,13 +9394,13 @@
         <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D13" t="s">
         <v>31</v>
       </c>
       <c r="E13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F13" t="s">
         <v>18</v>
@@ -9427,19 +9424,19 @@
         <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D14" t="s">
         <v>15</v>
       </c>
       <c r="E14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F14" t="s">
+        <v>106</v>
+      </c>
+      <c r="G14" s="8" t="s">
         <v>107</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>108</v>
       </c>
       <c r="I14" t="s">
         <v>40</v>
@@ -9448,7 +9445,7 @@
         <v>420</v>
       </c>
       <c r="L14" s="30" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
@@ -9459,13 +9456,13 @@
         <v>43</v>
       </c>
       <c r="C15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D15" t="s">
         <v>15</v>
       </c>
       <c r="E15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F15" t="s">
         <v>18</v>
@@ -9480,7 +9477,7 @@
         <v>0</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
@@ -9491,19 +9488,19 @@
         <v>43</v>
       </c>
       <c r="C16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D16" t="s">
         <v>15</v>
       </c>
       <c r="E16" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F16" t="s">
+        <v>106</v>
+      </c>
+      <c r="G16" s="8" t="s">
         <v>107</v>
-      </c>
-      <c r="G16" s="8" t="s">
-        <v>108</v>
       </c>
       <c r="I16" t="s">
         <v>40</v>
@@ -9521,28 +9518,28 @@
         <v>77</v>
       </c>
       <c r="C17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D17" t="s">
         <v>15</v>
       </c>
       <c r="E17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F17" t="s">
+        <v>106</v>
+      </c>
+      <c r="G17" t="s">
         <v>107</v>
       </c>
-      <c r="G17" t="s">
-        <v>108</v>
-      </c>
       <c r="I17" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J17">
         <v>42.5</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -9553,28 +9550,28 @@
         <v>77</v>
       </c>
       <c r="C18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D18" t="s">
         <v>15</v>
       </c>
       <c r="E18" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F18" t="s">
+        <v>106</v>
+      </c>
+      <c r="G18" t="s">
         <v>107</v>
       </c>
-      <c r="G18" t="s">
-        <v>108</v>
-      </c>
       <c r="I18" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J18">
         <v>0.125</v>
       </c>
       <c r="L18" s="30" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
@@ -9585,13 +9582,13 @@
         <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D19" t="s">
         <v>15</v>
       </c>
       <c r="E19" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F19" t="s">
         <v>18</v>
@@ -9606,7 +9603,7 @@
         <v>0</v>
       </c>
       <c r="L19" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
@@ -9617,13 +9614,13 @@
         <v>43</v>
       </c>
       <c r="C20" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D20" t="s">
         <v>15</v>
       </c>
       <c r="E20" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F20" t="s">
         <v>18</v>
@@ -9638,7 +9635,7 @@
         <v>0</v>
       </c>
       <c r="L20" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
@@ -9649,13 +9646,13 @@
         <v>77</v>
       </c>
       <c r="C21" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D21" t="s">
         <v>15</v>
       </c>
       <c r="E21" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F21" t="s">
         <v>18</v>
@@ -9667,7 +9664,7 @@
         <v>0.8</v>
       </c>
       <c r="L21" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.2">
@@ -9678,13 +9675,13 @@
         <v>77</v>
       </c>
       <c r="C22" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D22" t="s">
         <v>15</v>
       </c>
       <c r="E22" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F22" t="s">
         <v>18</v>
@@ -9696,7 +9693,7 @@
         <v>0.8</v>
       </c>
       <c r="L22" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
@@ -9707,13 +9704,13 @@
         <v>14</v>
       </c>
       <c r="C23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D23" t="s">
         <v>15</v>
       </c>
       <c r="E23" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F23" t="s">
         <v>18</v>
@@ -9725,7 +9722,7 @@
         <v>0.8</v>
       </c>
       <c r="L23" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -9736,13 +9733,13 @@
         <v>77</v>
       </c>
       <c r="C24" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D24" t="s">
         <v>15</v>
       </c>
       <c r="E24" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F24" t="s">
         <v>18</v>
@@ -9754,7 +9751,7 @@
         <v>0.8</v>
       </c>
       <c r="L24" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -9765,13 +9762,13 @@
         <v>77</v>
       </c>
       <c r="C25" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D25" t="s">
         <v>15</v>
       </c>
       <c r="E25" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F25" t="s">
         <v>18</v>
@@ -9783,7 +9780,7 @@
         <v>0.8</v>
       </c>
       <c r="L25" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
@@ -9794,13 +9791,13 @@
         <v>14</v>
       </c>
       <c r="C26" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D26" t="s">
         <v>15</v>
       </c>
       <c r="E26" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F26" t="s">
         <v>18</v>
@@ -9815,7 +9812,7 @@
         <v>0</v>
       </c>
       <c r="L26" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
@@ -9826,19 +9823,19 @@
         <v>14</v>
       </c>
       <c r="C27" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D27" t="s">
         <v>15</v>
       </c>
       <c r="E27" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F27" t="s">
+        <v>106</v>
+      </c>
+      <c r="G27" t="s">
         <v>107</v>
-      </c>
-      <c r="G27" t="s">
-        <v>108</v>
       </c>
       <c r="I27" t="s">
         <v>40</v>
@@ -9855,13 +9852,13 @@
         <v>14</v>
       </c>
       <c r="C28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D28" t="s">
         <v>15</v>
       </c>
       <c r="E28" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F28" t="s">
         <v>18</v>
@@ -9873,7 +9870,7 @@
         <v>0.8</v>
       </c>
       <c r="L28" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -10080,22 +10077,22 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>96</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>2</v>
@@ -10111,30 +10108,30 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D4" t="s">
         <v>120</v>
       </c>
-      <c r="B4" t="s">
-        <v>103</v>
-      </c>
-      <c r="C4" t="s">
-        <v>103</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>121</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
+        <v>120</v>
+      </c>
+      <c r="G4" t="s">
         <v>122</v>
-      </c>
-      <c r="F4" t="s">
-        <v>121</v>
-      </c>
-      <c r="G4" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B5" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$2:$A$980, B$1,  'Country Extraction'!$B$2:$B$980, "All",  'Country Extraction'!$C$2:$C$980, $A5) = 0, "Missing", "Complete")</f>
@@ -10163,7 +10160,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B6" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$2:$A$980, B$1,  'Country Extraction'!$B$2:$B$980, "All",  'Country Extraction'!$C$2:$C$980, $A6) = 0, "Missing", "Complete")</f>
@@ -10192,226 +10189,226 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D7" t="s">
+        <v>120</v>
+      </c>
+      <c r="E7" t="s">
         <v>121</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
+        <v>120</v>
+      </c>
+      <c r="G7" t="s">
         <v>122</v>
-      </c>
-      <c r="F7" t="s">
-        <v>121</v>
-      </c>
-      <c r="G7" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D8" t="s">
+        <v>120</v>
+      </c>
+      <c r="E8" t="s">
         <v>121</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
+        <v>120</v>
+      </c>
+      <c r="G8" t="s">
         <v>122</v>
-      </c>
-      <c r="F8" t="s">
-        <v>121</v>
-      </c>
-      <c r="G8" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C9" t="s">
+        <v>102</v>
+      </c>
+      <c r="D9" t="s">
+        <v>120</v>
+      </c>
+      <c r="E9" t="s">
+        <v>121</v>
+      </c>
+      <c r="F9" t="s">
+        <v>120</v>
+      </c>
+      <c r="G9" t="s">
+        <v>122</v>
+      </c>
+      <c r="H9" t="s">
         <v>128</v>
-      </c>
-      <c r="B9" t="s">
-        <v>103</v>
-      </c>
-      <c r="C9" t="s">
-        <v>103</v>
-      </c>
-      <c r="D9" t="s">
-        <v>121</v>
-      </c>
-      <c r="E9" t="s">
-        <v>122</v>
-      </c>
-      <c r="F9" t="s">
-        <v>121</v>
-      </c>
-      <c r="G9" t="s">
-        <v>123</v>
-      </c>
-      <c r="H9" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E10" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, F$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A10, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="F10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G10" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, H$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A10, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E11" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, F$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A11, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="F11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D12" t="s">
+        <v>120</v>
+      </c>
+      <c r="E12" t="s">
         <v>121</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
+        <v>120</v>
+      </c>
+      <c r="G12" t="s">
         <v>122</v>
-      </c>
-      <c r="F12" t="s">
-        <v>121</v>
-      </c>
-      <c r="G12" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>134</v>
+      </c>
+      <c r="B13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C13" t="s">
+        <v>102</v>
+      </c>
+      <c r="D13" t="s">
+        <v>120</v>
+      </c>
+      <c r="E13" t="s">
+        <v>121</v>
+      </c>
+      <c r="F13" t="s">
+        <v>120</v>
+      </c>
+      <c r="G13" t="s">
+        <v>122</v>
+      </c>
+      <c r="H13" t="s">
         <v>135</v>
-      </c>
-      <c r="B13" t="s">
-        <v>103</v>
-      </c>
-      <c r="C13" t="s">
-        <v>103</v>
-      </c>
-      <c r="D13" t="s">
-        <v>121</v>
-      </c>
-      <c r="E13" t="s">
-        <v>122</v>
-      </c>
-      <c r="F13" t="s">
-        <v>121</v>
-      </c>
-      <c r="G13" t="s">
-        <v>123</v>
-      </c>
-      <c r="H13" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>136</v>
+      </c>
+      <c r="B14" t="s">
+        <v>102</v>
+      </c>
+      <c r="C14" t="s">
+        <v>102</v>
+      </c>
+      <c r="D14" t="s">
+        <v>120</v>
+      </c>
+      <c r="E14" t="s">
+        <v>121</v>
+      </c>
+      <c r="F14" t="s">
+        <v>120</v>
+      </c>
+      <c r="G14" t="s">
+        <v>122</v>
+      </c>
+      <c r="H14" t="s">
         <v>137</v>
-      </c>
-      <c r="B14" t="s">
-        <v>103</v>
-      </c>
-      <c r="C14" t="s">
-        <v>103</v>
-      </c>
-      <c r="D14" t="s">
-        <v>121</v>
-      </c>
-      <c r="E14" t="s">
-        <v>122</v>
-      </c>
-      <c r="F14" t="s">
-        <v>121</v>
-      </c>
-      <c r="G14" t="s">
-        <v>123</v>
-      </c>
-      <c r="H14" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C15" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, D$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A15, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="D15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E15" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, F$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A15, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="F15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G15" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, H$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A15, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
@@ -10482,19 +10479,19 @@
         <v>13</v>
       </c>
       <c r="B2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C2" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="E2" t="s">
         <v>141</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
+        <v>141</v>
+      </c>
+      <c r="J2" s="11" t="s">
         <v>142</v>
-      </c>
-      <c r="G2" t="s">
-        <v>142</v>
-      </c>
-      <c r="J2" s="11" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -10505,16 +10502,16 @@
         <v>27</v>
       </c>
       <c r="C3" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E3" t="s">
         <v>141</v>
       </c>
-      <c r="E3" t="s">
-        <v>142</v>
-      </c>
       <c r="G3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J3" s="13" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
@@ -10525,13 +10522,13 @@
         <v>28</v>
       </c>
       <c r="C4" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E4" t="s">
         <v>141</v>
       </c>
-      <c r="E4" t="s">
-        <v>142</v>
-      </c>
       <c r="G4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
@@ -10542,13 +10539,13 @@
         <v>29</v>
       </c>
       <c r="C5" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E5" t="s">
         <v>141</v>
       </c>
-      <c r="E5" t="s">
-        <v>142</v>
-      </c>
       <c r="G5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
@@ -10559,13 +10556,13 @@
         <v>30</v>
       </c>
       <c r="C6" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E6" t="s">
         <v>141</v>
       </c>
-      <c r="E6" t="s">
-        <v>142</v>
-      </c>
       <c r="G6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
@@ -10576,115 +10573,115 @@
         <v>31</v>
       </c>
       <c r="C7" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E7" t="s">
         <v>141</v>
       </c>
-      <c r="E7" t="s">
-        <v>142</v>
-      </c>
       <c r="G7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="E8" t="s">
         <v>141</v>
       </c>
-      <c r="E8" t="s">
-        <v>142</v>
-      </c>
       <c r="G8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B9" t="s">
         <v>27</v>
       </c>
       <c r="C9" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E9" t="s">
         <v>141</v>
       </c>
-      <c r="E9" t="s">
-        <v>142</v>
-      </c>
       <c r="G9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B10" t="s">
         <v>28</v>
       </c>
       <c r="C10" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E10" t="s">
         <v>141</v>
       </c>
-      <c r="E10" t="s">
-        <v>142</v>
-      </c>
       <c r="G10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B11" t="s">
         <v>29</v>
       </c>
       <c r="C11" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E11" t="s">
         <v>141</v>
       </c>
-      <c r="E11" t="s">
-        <v>142</v>
-      </c>
       <c r="G11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B12" t="s">
         <v>30</v>
       </c>
       <c r="C12" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E12" t="s">
         <v>141</v>
       </c>
-      <c r="E12" t="s">
-        <v>142</v>
-      </c>
       <c r="G12" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B13" t="s">
         <v>31</v>
       </c>
       <c r="C13" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E13" t="s">
         <v>141</v>
       </c>
-      <c r="E13" t="s">
-        <v>142</v>
-      </c>
       <c r="G13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
@@ -10692,16 +10689,16 @@
         <v>76</v>
       </c>
       <c r="B14" t="s">
+        <v>139</v>
+      </c>
+      <c r="C14" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="E14" t="s">
         <v>141</v>
       </c>
-      <c r="E14" t="s">
-        <v>142</v>
-      </c>
       <c r="G14" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
@@ -10712,13 +10709,13 @@
         <v>27</v>
       </c>
       <c r="C15" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E15" t="s">
         <v>141</v>
       </c>
-      <c r="E15" t="s">
-        <v>142</v>
-      </c>
       <c r="G15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
@@ -10729,13 +10726,13 @@
         <v>28</v>
       </c>
       <c r="C16" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E16" t="s">
         <v>141</v>
       </c>
-      <c r="E16" t="s">
-        <v>142</v>
-      </c>
       <c r="G16" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
@@ -10746,13 +10743,13 @@
         <v>29</v>
       </c>
       <c r="C17" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E17" t="s">
         <v>141</v>
       </c>
-      <c r="E17" t="s">
-        <v>142</v>
-      </c>
       <c r="G17" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
@@ -10763,13 +10760,13 @@
         <v>30</v>
       </c>
       <c r="C18" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E18" t="s">
         <v>141</v>
       </c>
-      <c r="E18" t="s">
-        <v>142</v>
-      </c>
       <c r="G18" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
@@ -10780,13 +10777,13 @@
         <v>31</v>
       </c>
       <c r="C19" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E19" t="s">
         <v>141</v>
       </c>
-      <c r="E19" t="s">
-        <v>142</v>
-      </c>
       <c r="G19" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -10794,19 +10791,19 @@
         <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C20" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E20" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="G20" t="s">
+        <v>141</v>
+      </c>
+      <c r="J20" s="11" t="s">
         <v>147</v>
-      </c>
-      <c r="G20" t="s">
-        <v>142</v>
-      </c>
-      <c r="J20" s="11" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
@@ -10817,16 +10814,16 @@
         <v>27</v>
       </c>
       <c r="C21" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E21" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E21" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G21" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
@@ -10837,13 +10834,13 @@
         <v>28</v>
       </c>
       <c r="C22" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E22" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E22" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G22" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
@@ -10854,13 +10851,13 @@
         <v>29</v>
       </c>
       <c r="C23" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E23" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E23" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G23" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
@@ -10871,13 +10868,13 @@
         <v>30</v>
       </c>
       <c r="C24" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E24" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E24" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G24" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
@@ -10888,115 +10885,115 @@
         <v>31</v>
       </c>
       <c r="C25" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E25" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E25" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G25" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
+        <v>144</v>
+      </c>
+      <c r="B26" t="s">
+        <v>139</v>
+      </c>
+      <c r="C26" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="B26" t="s">
-        <v>140</v>
-      </c>
-      <c r="C26" s="9" t="s">
+      <c r="E26" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E26" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G26" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B27" t="s">
         <v>27</v>
       </c>
       <c r="C27" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E27" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E27" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G27" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B28" t="s">
         <v>28</v>
       </c>
       <c r="C28" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E28" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E28" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G28" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B29" t="s">
         <v>29</v>
       </c>
       <c r="C29" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E29" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E29" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G29" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B30" t="s">
         <v>30</v>
       </c>
       <c r="C30" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E30" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E30" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G30" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B31" t="s">
         <v>31</v>
       </c>
       <c r="C31" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E31" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E31" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
@@ -11004,16 +11001,16 @@
         <v>76</v>
       </c>
       <c r="B32" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C32" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E32" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E32" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G32" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
@@ -11024,13 +11021,13 @@
         <v>27</v>
       </c>
       <c r="C33" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E33" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E33" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G33" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
@@ -11041,13 +11038,13 @@
         <v>28</v>
       </c>
       <c r="C34" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E34" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E34" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G34" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
@@ -11058,13 +11055,13 @@
         <v>29</v>
       </c>
       <c r="C35" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E35" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E35" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G35" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
@@ -11075,13 +11072,13 @@
         <v>30</v>
       </c>
       <c r="C36" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E36" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E36" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G36" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
@@ -11092,13 +11089,13 @@
         <v>31</v>
       </c>
       <c r="C37" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E37" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E37" s="8" t="s">
-        <v>147</v>
-      </c>
       <c r="G37" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
@@ -11106,13 +11103,13 @@
         <v>13</v>
       </c>
       <c r="B38" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C38" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="G38" s="9" t="s">
         <v>149</v>
-      </c>
-      <c r="G38" s="9" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
@@ -11123,10 +11120,10 @@
         <v>27</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
@@ -11137,10 +11134,10 @@
         <v>28</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
@@ -11151,10 +11148,10 @@
         <v>29</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
@@ -11165,10 +11162,10 @@
         <v>30</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -11179,94 +11176,94 @@
         <v>31</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B44" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B45" t="s">
         <v>27</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G45" s="14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B46" t="s">
         <v>28</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B47" t="s">
         <v>29</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G47" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B48" t="s">
         <v>30</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G48" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B49" t="s">
         <v>31</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G49" s="14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
@@ -11274,13 +11271,13 @@
         <v>76</v>
       </c>
       <c r="B50" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.2">
@@ -11291,10 +11288,10 @@
         <v>27</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G51" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
@@ -11305,10 +11302,10 @@
         <v>28</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G52" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.2">
@@ -11319,10 +11316,10 @@
         <v>29</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G53" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.2">
@@ -11333,10 +11330,10 @@
         <v>30</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G54" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
@@ -11347,10 +11344,10 @@
         <v>31</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G55" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.2">
@@ -11358,13 +11355,13 @@
         <v>13</v>
       </c>
       <c r="B56" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C56" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G56" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -11375,10 +11372,10 @@
         <v>27</v>
       </c>
       <c r="C57" t="s">
+        <v>155</v>
+      </c>
+      <c r="J57" s="13" t="s">
         <v>156</v>
-      </c>
-      <c r="J57" s="13" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -11389,10 +11386,10 @@
         <v>28</v>
       </c>
       <c r="C58" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J58" s="12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -11403,7 +11400,7 @@
         <v>29</v>
       </c>
       <c r="C59" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J59" s="12"/>
     </row>
@@ -11415,7 +11412,7 @@
         <v>30</v>
       </c>
       <c r="C60" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.2">
@@ -11426,76 +11423,76 @@
         <v>31</v>
       </c>
       <c r="C61" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B62" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C62" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G62" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B63" t="s">
         <v>27</v>
       </c>
       <c r="C63" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B64" t="s">
         <v>28</v>
       </c>
       <c r="C64" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B65" t="s">
         <v>29</v>
       </c>
       <c r="C65" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B66" t="s">
         <v>30</v>
       </c>
       <c r="C66" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B67" t="s">
         <v>31</v>
       </c>
       <c r="C67" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.2">
@@ -11503,13 +11500,13 @@
         <v>76</v>
       </c>
       <c r="B68" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C68" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G68" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.2">
@@ -11520,7 +11517,7 @@
         <v>27</v>
       </c>
       <c r="C69" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.2">
@@ -11531,7 +11528,7 @@
         <v>28</v>
       </c>
       <c r="C70" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.2">
@@ -11542,7 +11539,7 @@
         <v>29</v>
       </c>
       <c r="C71" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.2">
@@ -11553,7 +11550,7 @@
         <v>30</v>
       </c>
       <c r="C72" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.2">
@@ -11564,7 +11561,7 @@
         <v>31</v>
       </c>
       <c r="C73" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="74" spans="1:10" ht="29.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -11572,36 +11569,36 @@
         <v>13</v>
       </c>
       <c r="B74" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C74" t="s">
+        <v>158</v>
+      </c>
+      <c r="D74" t="s">
         <v>159</v>
       </c>
-      <c r="D74" t="s">
+      <c r="G74" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="G74" s="12" t="s">
+      <c r="J74" s="14" t="s">
         <v>161</v>
-      </c>
-      <c r="J74" s="14" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B75" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C75" t="s">
+        <v>158</v>
+      </c>
+      <c r="D75" t="s">
         <v>159</v>
       </c>
-      <c r="D75" t="s">
-        <v>160</v>
-      </c>
       <c r="J75" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.2">
@@ -11609,13 +11606,13 @@
         <v>76</v>
       </c>
       <c r="B76" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C76" t="s">
+        <v>158</v>
+      </c>
+      <c r="D76" t="s">
         <v>159</v>
-      </c>
-      <c r="D76" t="s">
-        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -11682,10 +11679,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C3" t="str">
         <f>IF(COUNTIFS('Vehicle Extraction'!$A$2:$A$904, C$1,  'Vehicle Extraction'!$B$2:$B$904, $A3) = 0, "Missing", "Complete")</f>
@@ -11698,10 +11695,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="26" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C4" t="str">
         <f>IF(COUNTIFS('Vehicle Extraction'!$A$2:$A$904, C$1,  'Vehicle Extraction'!$B$2:$B$904, $A4) = 0, "Missing", "Complete")</f>
@@ -11770,28 +11767,28 @@
         <v>77</v>
       </c>
       <c r="B2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D2" t="s">
         <v>166</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>167</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" s="5" t="s">
         <v>168</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>169</v>
       </c>
       <c r="G2" s="26">
         <v>3.25</v>
       </c>
       <c r="H2" s="26" t="s">
+        <v>169</v>
+      </c>
+      <c r="I2" s="5" t="s">
         <v>170</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -11799,28 +11796,28 @@
         <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D3" t="s">
         <v>166</v>
-      </c>
-      <c r="D3" t="s">
-        <v>167</v>
       </c>
       <c r="E3">
         <v>2021</v>
       </c>
       <c r="F3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G3">
         <v>4.4000000000000004</v>
       </c>
       <c r="H3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I3" s="6" t="s">
         <v>173</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -11828,28 +11825,28 @@
         <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D4" t="s">
         <v>166</v>
-      </c>
-      <c r="D4" t="s">
-        <v>167</v>
       </c>
       <c r="E4">
         <v>2012</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G4">
         <v>4.2</v>
       </c>
       <c r="H4" t="s">
+        <v>175</v>
+      </c>
+      <c r="I4" s="6" t="s">
         <v>176</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -11857,28 +11854,28 @@
         <v>77</v>
       </c>
       <c r="B5" t="s">
+        <v>164</v>
+      </c>
+      <c r="C5" t="s">
         <v>165</v>
       </c>
-      <c r="C5" t="s">
-        <v>166</v>
-      </c>
       <c r="D5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E5">
         <v>2013</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G5">
         <v>1.67</v>
       </c>
       <c r="H5" t="s">
+        <v>179</v>
+      </c>
+      <c r="I5" s="6" t="s">
         <v>180</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -11886,28 +11883,28 @@
         <v>43</v>
       </c>
       <c r="B6" t="s">
+        <v>164</v>
+      </c>
+      <c r="C6" t="s">
         <v>165</v>
       </c>
-      <c r="C6" t="s">
-        <v>166</v>
-      </c>
       <c r="D6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E6">
         <v>2013</v>
       </c>
       <c r="F6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G6">
         <v>1.67</v>
       </c>
       <c r="H6" t="s">
+        <v>179</v>
+      </c>
+      <c r="I6" s="6" t="s">
         <v>180</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="115.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -12032,7 +12029,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="26" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -12045,59 +12042,59 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="26" t="s">
+        <v>182</v>
+      </c>
+      <c r="B3" s="26" t="s">
         <v>183</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="C3" s="26" t="s">
         <v>184</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>185</v>
       </c>
       <c r="D3" s="26">
         <v>2018</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F3" s="26">
         <v>4.3</v>
       </c>
       <c r="G3" s="26" t="s">
+        <v>186</v>
+      </c>
+      <c r="H3" s="24" t="s">
         <v>187</v>
-      </c>
-      <c r="H3" s="24" t="s">
-        <v>188</v>
       </c>
       <c r="I3" s="23"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="26" t="s">
+        <v>188</v>
+      </c>
+      <c r="B4" s="26" t="s">
         <v>189</v>
       </c>
-      <c r="B4" s="26" t="s">
+      <c r="C4" s="26" t="s">
         <v>190</v>
-      </c>
-      <c r="C4" s="26" t="s">
-        <v>191</v>
       </c>
       <c r="D4" s="26">
         <v>2015</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F4" s="26">
         <v>6</v>
       </c>
       <c r="G4" s="27" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H4" s="23"/>
       <c r="I4" s="23"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="26" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
@@ -12110,18 +12107,18 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="26" t="s">
+        <v>194</v>
+      </c>
+      <c r="B6" s="26" t="s">
         <v>195</v>
-      </c>
-      <c r="B6" s="26" t="s">
-        <v>196</v>
       </c>
       <c r="C6" s="26"/>
       <c r="D6" s="26"/>
       <c r="E6" s="26" t="s">
+        <v>196</v>
+      </c>
+      <c r="F6" s="26" t="s">
         <v>197</v>
-      </c>
-      <c r="F6" s="26" t="s">
-        <v>198</v>
       </c>
       <c r="G6" s="26"/>
       <c r="H6" s="23"/>
@@ -12129,18 +12126,18 @@
     </row>
     <row r="7" spans="1:9" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="26" t="s">
+        <v>194</v>
+      </c>
+      <c r="B7" s="26" t="s">
         <v>195</v>
-      </c>
-      <c r="B7" s="26" t="s">
-        <v>196</v>
       </c>
       <c r="C7" s="26"/>
       <c r="D7" s="26"/>
       <c r="E7" s="26" t="s">
+        <v>198</v>
+      </c>
+      <c r="F7" s="31" t="s">
         <v>199</v>
-      </c>
-      <c r="F7" s="31" t="s">
-        <v>200</v>
       </c>
       <c r="G7" s="26"/>
       <c r="H7" s="23"/>
@@ -12148,22 +12145,22 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="26" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C8" s="26"/>
       <c r="D8" s="26"/>
       <c r="E8" s="26" t="s">
+        <v>201</v>
+      </c>
+      <c r="F8" s="26" t="s">
         <v>202</v>
-      </c>
-      <c r="F8" s="26" t="s">
-        <v>203</v>
       </c>
       <c r="G8" s="26"/>
       <c r="H8" s="23" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="I8" s="23"/>
     </row>

</xml_diff>

<commit_message>
add Nigeria/folate/wheat with dummy data
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -1404,7 +1404,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="8" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2965,6 +2965,156 @@
       <c r="J31" s="43" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Intervention coverage % of fortifiable</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>DUMMY (SSCI-2784)</t>
+        </is>
+      </c>
+      <c r="I32" s="41" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (SSCI-2784): folate value copied from the corresponding Nigeria Rice Folate row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Intervention effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>DUMMY (SSCI-2784)</t>
+        </is>
+      </c>
+      <c r="I33" s="41" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (SSCI-2784): folate value copied from the corresponding Nigeria Rice Folate row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Vehicle fortification in intervention -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>DUMMY (SSCI-2784)</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="J34" s="43" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (SSCI-2784): folate value copied from the corresponding Nigeria Rice Folate row. Replace with real wheat data.</t>
         </is>
       </c>
     </row>
@@ -9635,7 +9785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="8" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -11001,6 +11151,156 @@
       <c r="L28" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- any</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>DUMMY (SSCI-2784)</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (SSCI-2784): folate value copied from the corresponding Nigeria Rice Folate row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>DUMMY (SSCI-2784)</t>
+        </is>
+      </c>
+      <c r="J30" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (SSCI-2784): folate value copied from the corresponding Nigeria Rice Folate row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Baseline effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>DUMMY (SSCI-2784)</t>
+        </is>
+      </c>
+      <c r="J31" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (SSCI-2784): folate value copied from the corresponding Nigeria Rice Folate row. Replace with real wheat data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Albrja/mic 7549/implement nigeria iron wheat (#45)
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -1404,7 +1404,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="8" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2818,6 +2818,156 @@
         </is>
       </c>
     </row>
+    <row r="29" ht="15" customHeight="1">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Intervention coverage % of fortifiable</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="I29" s="41" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Intervention effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="I30" s="41" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Vehicle fortification in intervention -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>40</v>
+      </c>
+      <c r="J31" s="43" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="4">
     <dataValidation sqref="A1:B1" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1"/>
@@ -2828,7 +2978,7 @@
       <formula1>"Iron,Folate"</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"Bouillon,Salt,Rice"</formula1>
+      <formula1>"Bouillon,Salt,Rice,Wheat"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -2973,7 +3123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M86"/>
+  <dimension ref="A1:M117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="8" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7408,10 +7558,1556 @@
         <v>0.676</v>
       </c>
     </row>
-    <row r="91" ht="15" customHeight="1"/>
-    <row r="92" ht="15" customHeight="1"/>
-    <row r="97" ht="15" customHeight="1"/>
-    <row r="102" ht="15" customHeight="1"/>
+    <row r="87" ht="15" customHeight="1">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Vehicle "fortifiability" (essentially amount industrially produced)</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J87" s="7" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="M87" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="43.5" customHeight="1">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J88" t="n">
+        <v>32.803200000000004</v>
+      </c>
+      <c r="M88" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="43.5" customHeight="1">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J89" t="n">
+        <v>11.491200000000001</v>
+      </c>
+      <c r="M89" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="43.5" customHeight="1">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J90" t="n">
+        <v>23.475200000000001</v>
+      </c>
+      <c r="M90" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="43.5" customHeight="1">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J91" t="n">
+        <v>33.142200000000003</v>
+      </c>
+      <c r="M91" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="43.5" customHeight="1">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J92" t="n">
+        <v>46.652100000000004</v>
+      </c>
+      <c r="M92" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="43.5" customHeight="1">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J93" t="n">
+        <v>53.742000000000004</v>
+      </c>
+      <c r="M93" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="29.25" customHeight="1">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J94" s="21" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="M94" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J95" s="21" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J96" s="21" t="n">
+        <v>0.448</v>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J97" s="21" t="n">
+        <v>0.546</v>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J98" s="21" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J99" s="21" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="29.25" customHeight="1">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J100" t="n">
+        <v>40.074074074074069</v>
+      </c>
+      <c r="M100" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J101" t="n">
+        <v>24.814814814814813</v>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J102" t="n">
+        <v>33.333333333333336</v>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J103" t="n">
+        <v>35.037037037037031</v>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J104" t="n">
+        <v>37.777777777777779</v>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J105" t="n">
+        <v>39.037037037037031</v>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="43.5" customHeight="1">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- amount</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J106" t="n">
+        <v>20.5288</v>
+      </c>
+      <c r="M106" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="43.5" customHeight="1">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- amount</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J107" t="n">
+        <v>19.028000000000002</v>
+      </c>
+      <c r="M107" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="43.5" customHeight="1">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- amount</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J108" t="n">
+        <v>21.976000000000003</v>
+      </c>
+      <c r="M108" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="29.25" customHeight="1">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- amount</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J109" t="n">
+        <v>25.62962962962963</v>
+      </c>
+      <c r="M109" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="29.25" customHeight="1">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- amount</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J110" t="n">
+        <v>23.999999999999996</v>
+      </c>
+      <c r="M110" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="29.25" customHeight="1">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- amount</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J111" t="n">
+        <v>27.333333333333336</v>
+      </c>
+      <c r="M111" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="29.25" customHeight="1">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- any</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J112" s="21" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="M112" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- any</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J113" s="21" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- any</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J114" s="21" t="n">
+        <v>0.448</v>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- any</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J115" s="21" t="n">
+        <v>0.546</v>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- any</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J116" s="21" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by U5 children -- any</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J117" s="21" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="5">
     <dataValidation sqref="A1:B1" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1"/>
@@ -7422,7 +9118,7 @@
       <formula1>"Nigeria,Ethiopia,India"</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"Bouillon,Salt,Rice"</formula1>
+      <formula1>"Bouillon,Salt,Rice,Wheat"</formula1>
     </dataValidation>
     <dataValidation sqref="D1:D1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"All (assumed same),Total,Female,Male"</formula1>
@@ -7939,7 +9635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="8" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9158,11 +10854,161 @@
         </is>
       </c>
     </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- any</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J27" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Baseline effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="J28" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="5">
     <dataValidation sqref="A1:B1" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1"/>
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"Bouillon,Salt,Rice"</formula1>
+      <formula1>"Bouillon,Salt,Rice,Wheat"</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Iron,Folate"</formula1>
@@ -11737,7 +13583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="8" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -12011,6 +13857,76 @@
       <c r="I6" s="6" t="inlineStr">
         <is>
           <t>https://www.bmj.com/content/346/bmj.f3443; study of supplementation at higher doses than fortification; selected the effect among trials &lt;66mg/day as all fortification would fall in this range</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="115.5" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Iron fortification/consumption effect on hemoglobin</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Mean difference</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>g/L</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="G7" s="26" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="43.5" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Iron fortification/consumption effect on birthweight</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Mean difference</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>g/(mg/person-day)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7549)</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement India wheat iron
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -2008,7 +2008,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -3255,6 +3255,156 @@
       <c s="39" r="J37" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Intervention coverage % of fortifiable</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="37" r="I38" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Intervention effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="37" r="I39" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Vehicle fortification in intervention -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>40</v>
+      </c>
+      <c r="J40" s="39" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
         </is>
       </c>
     </row>
@@ -3367,7 +3517,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M141"/>
+  <dimension ref="A1:M155"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -8597,6 +8747,706 @@
       <c r="M141" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Vehicle "fortifiability" (essentially amount industrially produced)</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="7" r="J142" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="M142" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J143" t="n">
+        <v>32.803200000000004</v>
+      </c>
+      <c r="M143" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J144" t="n">
+        <v>11.491200000000001</v>
+      </c>
+      <c r="M144" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J145" t="n">
+        <v>23.475200000000001</v>
+      </c>
+      <c r="M145" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J146" t="n">
+        <v>33.142200000000003</v>
+      </c>
+      <c r="M146" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J147" t="n">
+        <v>46.652100000000004</v>
+      </c>
+      <c r="M147" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J148" t="n">
+        <v>53.742000000000004</v>
+      </c>
+      <c r="M148" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" spans="1:13" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J149" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="M149" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J150" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J151" t="n">
+        <v>0.448</v>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J152" t="n">
+        <v>0.546</v>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J153" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J154" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" spans="1:13" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J155" t="n">
+        <v>40.074074074074069</v>
+      </c>
+      <c r="M155" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): Nigeria wheat WRA Total SD, applied to every quintile. Replace with real India wheat data.</t>
         </is>
       </c>
     </row>
@@ -8998,7 +9848,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -10020,6 +10870,156 @@
       <c r="L31" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- any</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c s="8" r="G32" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="7" r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c s="8" r="G33" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="10" r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Baseline effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c s="8" r="G34" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="7" r="J34" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add India/salt/iron with placeholder data (MIC-7580)
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -2008,7 +2008,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -3405,6 +3405,156 @@
       <c r="J40" s="39" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Intervention coverage % of fortifiable</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="37" r="I41" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Intervention effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="37" r="I42" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Vehicle fortification in intervention -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>40</v>
+      </c>
+      <c r="J43" s="39" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3667,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M155"/>
+  <dimension ref="A1:M169"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -9447,6 +9597,706 @@
       <c r="M155" s="5" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7580): Nigeria wheat WRA Total SD, applied to every quintile. Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Vehicle "fortifiability" (essentially amount industrially produced)</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="7" r="J156" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="M156" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J157" t="n">
+        <v>32.803200000000004</v>
+      </c>
+      <c r="M157" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J158" t="n">
+        <v>11.491200000000001</v>
+      </c>
+      <c r="M158" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J159" t="n">
+        <v>23.475200000000001</v>
+      </c>
+      <c r="M159" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J160" t="n">
+        <v>33.142200000000003</v>
+      </c>
+      <c r="M160" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J161" t="n">
+        <v>46.652100000000004</v>
+      </c>
+      <c r="M161" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J162" t="n">
+        <v>53.742000000000004</v>
+      </c>
+      <c r="M162" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" spans="1:13" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J163" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="M163" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J164" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J165" t="n">
+        <v>0.448</v>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J166" t="n">
+        <v>0.546</v>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J167" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J168" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" spans="1:13" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J169" t="n">
+        <v>40.074074074074069</v>
+      </c>
+      <c r="M169" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
         </is>
       </c>
     </row>
@@ -9848,7 +10698,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -11020,6 +11870,156 @@
       <c r="L34" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- any</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c s="8" r="G35" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="7" r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c s="8" r="G36" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="10" r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Baseline effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c s="8" r="G37" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="7" r="J37" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
         </is>
       </c>
     </row>
@@ -12721,7 +13721,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -12974,6 +13974,41 @@
       <c s="6" r="I8" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Iron fortification/consumption effect on birthweight</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mean difference</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>g/(mg/person-day)</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): copied from the wheat row; every vehicle uses 1.67. Confirm for salt.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ndbs/nigeria folate wheat (#48)
* add Nigeria/folate/wheat with dummy data

* run data prep notebooks

* run NTD notebook for Nigeria/wheat
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -1404,7 +1404,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="8" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2965,6 +2965,156 @@
       <c r="J31" s="43" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Intervention coverage % of fortifiable</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>DUMMY (SSCI-2784)</t>
+        </is>
+      </c>
+      <c r="I32" s="41" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (SSCI-2784): folate value copied from the corresponding Nigeria Rice Folate row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Intervention effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>DUMMY (SSCI-2784)</t>
+        </is>
+      </c>
+      <c r="I33" s="41" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (SSCI-2784): folate value copied from the corresponding Nigeria Rice Folate row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Vehicle fortification in intervention -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>DUMMY (SSCI-2784)</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="J34" s="43" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (SSCI-2784): folate value copied from the corresponding Nigeria Rice Folate row. Replace with real wheat data.</t>
         </is>
       </c>
     </row>
@@ -9635,7 +9785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="8" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -11001,6 +11151,156 @@
       <c r="L28" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- any</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>DUMMY (SSCI-2784)</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (SSCI-2784): folate value copied from the corresponding Nigeria Rice Folate row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>DUMMY (SSCI-2784)</t>
+        </is>
+      </c>
+      <c r="J30" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (SSCI-2784): folate value copied from the corresponding Nigeria Rice Folate row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Baseline effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>DUMMY (SSCI-2784)</t>
+        </is>
+      </c>
+      <c r="J31" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (SSCI-2784): folate value copied from the corresponding Nigeria Rice Folate row. Replace with real wheat data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Albrja/mic 7580/india wheat iron (#50)
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -2008,7 +2008,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -3405,6 +3405,156 @@
       <c r="J40" s="39" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (SSCI-2784): folate value copied from the corresponding Nigeria Rice Folate row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Intervention coverage % of fortifiable</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="37" r="I41" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Intervention effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="37" r="I42" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Vehicle fortification in intervention -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>40</v>
+      </c>
+      <c r="J43" s="39" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3667,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M141"/>
+  <dimension ref="A1:M155"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -8747,6 +8897,706 @@
       <c r="M141" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Vehicle "fortifiability" (essentially amount industrially produced)</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="7" r="J142" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="M142" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J143" t="n">
+        <v>32.803200000000004</v>
+      </c>
+      <c r="M143" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J144" t="n">
+        <v>11.491200000000001</v>
+      </c>
+      <c r="M144" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J145" t="n">
+        <v>23.475200000000001</v>
+      </c>
+      <c r="M145" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J146" t="n">
+        <v>33.142200000000003</v>
+      </c>
+      <c r="M146" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J147" t="n">
+        <v>46.652100000000004</v>
+      </c>
+      <c r="M147" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J148" t="n">
+        <v>53.742000000000004</v>
+      </c>
+      <c r="M148" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" spans="1:13" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J149" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="M149" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J150" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J151" t="n">
+        <v>0.448</v>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J152" t="n">
+        <v>0.546</v>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J153" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J154" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" spans="1:13" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J155" t="n">
+        <v>40.074074074074069</v>
+      </c>
+      <c r="M155" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): Nigeria wheat WRA Total SD, applied to every quintile. Replace with real India wheat data.</t>
         </is>
       </c>
     </row>
@@ -9148,7 +9998,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -10320,6 +11170,156 @@
       <c r="L34" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (SSCI-2784): folate value copied from the corresponding Nigeria Rice Folate row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- any</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c s="8" r="G35" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="7" r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c s="8" r="G36" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="10" r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Baseline effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c s="8" r="G37" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="7" r="J37" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Ethiopia/wheat/folic acid with placeholder data (MIC-7585)
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -2008,7 +2008,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -3705,6 +3705,156 @@
       <c r="J46" s="39" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Intervention coverage % of fortifiable</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="I47" s="37" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Intervention effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="I48" s="37" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Vehicle fortification in intervention -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="J49" s="39" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real Ethiopia wheat data.</t>
         </is>
       </c>
     </row>
@@ -3817,7 +3967,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M169"/>
+  <dimension ref="A1:M183"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -10447,6 +10597,706 @@
       <c r="M169" s="5" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Vehicle "fortifiability" (essentially amount industrially produced)</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c s="7" r="J170" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="M170" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J171" t="n">
+        <v>32.803200000000004</v>
+      </c>
+      <c r="M171" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J172" t="n">
+        <v>11.491200000000001</v>
+      </c>
+      <c r="M172" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J173" t="n">
+        <v>23.475200000000001</v>
+      </c>
+      <c r="M173" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J174" t="n">
+        <v>33.142200000000003</v>
+      </c>
+      <c r="M174" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J175" t="n">
+        <v>46.652100000000004</v>
+      </c>
+      <c r="M175" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J176" t="n">
+        <v>53.742000000000004</v>
+      </c>
+      <c r="M176" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" spans="1:13" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c s="21" r="J177" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="M177" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c s="21" r="J178" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c s="21" r="J179" t="n">
+        <v>0.448</v>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c s="21" r="J180" t="n">
+        <v>0.546</v>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c s="21" r="J181" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c s="21" r="J182" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" spans="1:13" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J183" t="n">
+        <v>40.074074074074069</v>
+      </c>
+      <c r="M183" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
         </is>
       </c>
     </row>
@@ -10848,7 +11698,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -12320,6 +13170,156 @@
       <c r="L40" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- any</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J42" s="10" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Baseline effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J43" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real Ethiopia wheat data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add folic acid to India/wheat with placeholder data (MIC-7585)
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -2008,7 +2008,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -3855,6 +3855,156 @@
       <c r="J49" s="39" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Intervention coverage % of fortifiable</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="I50" s="37" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Intervention effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="I51" s="37" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Vehicle fortification in intervention -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="J52" s="39" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real India wheat data.</t>
         </is>
       </c>
     </row>
@@ -11698,7 +11848,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -13320,6 +13470,156 @@
       <c r="L43" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- any</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J44" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J45" s="10" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Baseline effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J46" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real India wheat data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Albrja/mic 7580/india salt iron (#51)
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -2008,7 +2008,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -3555,6 +3555,156 @@
       <c r="J43" s="39" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Intervention coverage % of fortifiable</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="37" r="I44" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Intervention effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="37" r="I45" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Vehicle fortification in intervention -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>40</v>
+      </c>
+      <c r="J46" s="39" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
         </is>
       </c>
     </row>
@@ -3667,7 +3817,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M155"/>
+  <dimension ref="A1:M169"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -9597,6 +9747,706 @@
       <c r="M155" s="5" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7580): Nigeria wheat WRA Total SD, applied to every quintile. Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Vehicle "fortifiability" (essentially amount industrially produced)</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="7" r="J156" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="M156" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J157" t="n">
+        <v>32.803200000000004</v>
+      </c>
+      <c r="M157" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J158" t="n">
+        <v>11.491200000000001</v>
+      </c>
+      <c r="M158" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J159" t="n">
+        <v>23.475200000000001</v>
+      </c>
+      <c r="M159" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J160" t="n">
+        <v>33.142200000000003</v>
+      </c>
+      <c r="M160" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J161" t="n">
+        <v>46.652100000000004</v>
+      </c>
+      <c r="M161" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J162" t="n">
+        <v>53.742000000000004</v>
+      </c>
+      <c r="M162" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" spans="1:13" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J163" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="M163" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J164" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J165" t="n">
+        <v>0.448</v>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J166" t="n">
+        <v>0.546</v>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J167" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="21" r="J168" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" spans="1:13" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="J169" t="n">
+        <v>40.074074074074069</v>
+      </c>
+      <c r="M169" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
         </is>
       </c>
     </row>
@@ -9998,7 +10848,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -11320,6 +12170,156 @@
       <c r="L37" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the Nigeria wheat placeholder row (itself copied from Nigeria rice). Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- any</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c s="8" r="G38" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="7" r="J38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c s="8" r="G39" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="10" r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Baseline effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c s="8" r="G40" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c s="7" r="J40" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
         </is>
       </c>
     </row>
@@ -13021,7 +14021,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -13274,6 +14274,41 @@
       <c s="6" r="I8" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7549): value copied from the corresponding Rice row. Replace with real wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Iron fortification/consumption effect on birthweight</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mean difference</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>g/(mg/person-day)</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7580)</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7580): copied from the wheat row; every vehicle uses 1.67. Confirm for salt.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Albrja/mic 7585/India and Ethiopia wheat folate (#52)
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -2008,7 +2008,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -3705,6 +3705,306 @@
       <c r="J46" s="39" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Intervention coverage % of fortifiable</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="I47" s="37" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Intervention effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="I48" s="37" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Vehicle fortification in intervention -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="J49" s="39" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Intervention coverage % of fortifiable</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="I50" s="37" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Intervention effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="I51" s="37" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Intervention</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Vehicle fortification in intervention -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="J52" s="39" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real India wheat data.</t>
         </is>
       </c>
     </row>
@@ -3817,7 +4117,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M169"/>
+  <dimension ref="A1:M183"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -10447,6 +10747,706 @@
       <c r="M169" s="5" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Vehicle "fortifiability" (essentially amount industrially produced)</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c s="7" r="J170" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="M170" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J171" t="n">
+        <v>32.803200000000004</v>
+      </c>
+      <c r="M171" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J172" t="n">
+        <v>11.491200000000001</v>
+      </c>
+      <c r="M172" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J173" t="n">
+        <v>23.475200000000001</v>
+      </c>
+      <c r="M173" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J174" t="n">
+        <v>33.142200000000003</v>
+      </c>
+      <c r="M174" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J175" t="n">
+        <v>46.652100000000004</v>
+      </c>
+      <c r="M175" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J176" t="n">
+        <v>53.742000000000004</v>
+      </c>
+      <c r="M176" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" spans="1:13" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c s="21" r="J177" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="M177" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c s="21" r="J178" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c s="21" r="J179" t="n">
+        <v>0.448</v>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c s="21" r="J180" t="n">
+        <v>0.546</v>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c s="21" r="J181" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- any</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c s="21" r="J182" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" spans="1:13" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Vehicle consumption by WRA -- amount</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>g/day</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J183" t="n">
+        <v>40.074074074074069</v>
+      </c>
+      <c r="M183" s="5" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the India wheat placeholder row. Replace with real Ethiopia wheat data.</t>
         </is>
       </c>
     </row>
@@ -10848,7 +11848,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -12320,6 +13320,306 @@
       <c r="L40" t="inlineStr">
         <is>
           <t>DUMMY PLACEHOLDER (MIC-7580): value copied from the India wheat placeholder row. Replace with real India salt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- any</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J42" s="10" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Baseline effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J43" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real Ethiopia wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- any</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J44" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Vehicle fortification at baseline -- amount among fortified</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>mcg/g</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J45" s="10" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real India wheat data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Baseline effective % of fortified</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>DUMMY (MIC-7585)</t>
+        </is>
+      </c>
+      <c r="J46" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>DUMMY PLACEHOLDER (MIC-7585): value copied from the Nigeria wheat folate placeholder row. Replace with real India wheat data.</t>
         </is>
       </c>
     </row>

</xml_diff>